<commit_message>
Order alphabetically for missing output
</commit_message>
<xml_diff>
--- a/unique_pairs.xlsx
+++ b/unique_pairs.xlsx
@@ -13,9 +13,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ge-La" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ir-Si" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gd-Si" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pt-Pt" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="La-Pt" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pt-Sb" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="La-Pt" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pt-Pt" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sb-Sb" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="La-Sb" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ce-Pt" sheetId="12" state="visible" r:id="rId12"/>
@@ -31,8 +31,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ge-Pt" sheetId="22" state="visible" r:id="rId22"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gd-Pt" sheetId="23" state="visible" r:id="rId23"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fe-Si" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Si-Si" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Si-Y" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Si-Y" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Si-Si" sheetId="26" state="visible" r:id="rId26"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ge-Tm" sheetId="27" state="visible" r:id="rId27"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dy-Pt" sheetId="28" state="visible" r:id="rId28"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Er-Ge" sheetId="29" state="visible" r:id="rId29"/>
@@ -1706,43 +1706,43 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>2.99</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Distance</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>300351.cif</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
         <v>2.242</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>File</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Distance</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>300351.cif</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>2.99</v>
       </c>
     </row>
   </sheetData>
@@ -2952,7 +2952,43 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Distance</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>300237.cif</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>3.14</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2997,18 +3033,28 @@
         <v>2.71</v>
       </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B5"/>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>300245.cif</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2.838</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3053,52 +3099,6 @@
         <v>2.71</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>300245.cif</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>2.838</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>File</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Distance</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>300237.cif</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>3.14</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>